<commit_message>
fix: Correct venue addresses and states in `venues.json` and update extracted quotes spreadsheets.
</commit_message>
<xml_diff>
--- a/Extracted_Quotes.xlsx
+++ b/Extracted_Quotes.xlsx
@@ -604,7 +604,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -614,7 +613,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>120 Exhibition St</t>
+          <t>120 Exhibition St, Melbourne VIC 3000</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -685,8 +684,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -947,8 +944,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -989,7 +984,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1025,8 +1019,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1157,7 +1149,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1288,7 +1279,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1374,7 +1364,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1685,7 +1674,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1726,7 +1714,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1767,7 +1754,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1803,8 +1789,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1845,7 +1829,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1900,7 +1883,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>101 Flinders Ln</t>
+          <t>101 Flinders Ln, Melbourne VIC 3000</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2021,7 +2004,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2031,7 +2013,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>15 Caxton St, Petrie Terrace, VIC 4000</t>
+          <t>15 Caxton St, Petrie Terrace, QLD 4000</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2057,7 +2039,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>x</t>
@@ -2103,7 +2084,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2189,7 +2169,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2545,7 +2524,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2631,7 +2609,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2672,7 +2649,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2758,7 +2734,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2844,7 +2819,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2880,8 +2854,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2917,8 +2889,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3004,7 +2974,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3220,8 +3189,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3352,7 +3319,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3433,8 +3399,6 @@
           <t>x</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: Standardize date formats and correct special characters in `venues.json`, and update `Extracted_Quotes.xlsx`.
</commit_message>
<xml_diff>
--- a/Extracted_Quotes.xlsx
+++ b/Extracted_Quotes.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcot./Documents/Australian-Venue/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C26BAE5E-B0DA-5444-B54A-2AAA6C254265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81CB1485-41A7-D147-AAA5-B15ABF02AC4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4420" yWindow="780" windowWidth="35360" windowHeight="25800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet!$A$1:$I$1</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -761,7 +764,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="d/mm/yyyy;@"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -770,12 +784,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -787,20 +807,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1108,7 +1128,7 @@
     <col min="2" max="2" width="44.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="48.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.5" bestFit="1" customWidth="1"/>
@@ -1116,31 +1136,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1157,7 +1177,7 @@
       <c r="D2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="2">
         <v>20579.939999999999</v>
       </c>
       <c r="F2" t="s">
@@ -1186,7 +1206,7 @@
       <c r="D3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="2">
         <v>17320</v>
       </c>
       <c r="F3" t="s">
@@ -1215,7 +1235,7 @@
       <c r="D4" s="1">
         <v>45972</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="2">
         <v>18658</v>
       </c>
       <c r="F4" t="s">
@@ -1241,7 +1261,7 @@
       <c r="D5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="2">
         <v>11571.52</v>
       </c>
       <c r="F5" t="s">
@@ -1270,7 +1290,7 @@
       <c r="D6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="2">
         <v>3242.15</v>
       </c>
       <c r="F6" t="s">
@@ -1293,7 +1313,7 @@
       <c r="D7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="2">
         <v>8364.14</v>
       </c>
       <c r="F7" t="s">
@@ -1322,7 +1342,7 @@
       <c r="D8" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="2">
         <v>12681.75</v>
       </c>
       <c r="F8" t="s">
@@ -1351,7 +1371,7 @@
       <c r="D9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="2">
         <v>17981.900000000001</v>
       </c>
       <c r="F9" t="s">
@@ -1380,7 +1400,7 @@
       <c r="D10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="2">
         <v>10694</v>
       </c>
       <c r="F10" t="s">
@@ -1409,7 +1429,7 @@
       <c r="D11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="2">
         <v>10431</v>
       </c>
       <c r="F11" t="s">
@@ -1438,7 +1458,7 @@
       <c r="D12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="2">
         <v>16157.15</v>
       </c>
       <c r="F12" t="s">
@@ -1461,7 +1481,7 @@
       <c r="D13" s="1">
         <v>45972</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="2">
         <v>13698.35</v>
       </c>
       <c r="F13" t="s">
@@ -1487,7 +1507,7 @@
       <c r="D14" s="1">
         <v>45972</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="2">
         <v>3733.4</v>
       </c>
       <c r="F14" t="s">
@@ -1510,7 +1530,7 @@
       <c r="D15" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="2">
         <v>11081.5</v>
       </c>
       <c r="F15" t="s">
@@ -1539,7 +1559,7 @@
       <c r="D16" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E16">
+      <c r="E16" s="2">
         <v>10217.4</v>
       </c>
       <c r="F16" t="s">
@@ -1568,7 +1588,7 @@
       <c r="D17" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="2">
         <v>21029.8</v>
       </c>
       <c r="F17" t="s">
@@ -1594,7 +1614,7 @@
       <c r="D18" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="2">
         <v>9708.0499999999993</v>
       </c>
       <c r="F18" t="s">
@@ -1623,7 +1643,7 @@
       <c r="D19" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E19">
+      <c r="E19" s="2">
         <v>5643.95</v>
       </c>
       <c r="F19" t="s">
@@ -1652,7 +1672,7 @@
       <c r="D20" s="1">
         <v>45972</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="2">
         <v>8902.9</v>
       </c>
       <c r="F20" t="s">
@@ -1678,7 +1698,7 @@
       <c r="D21" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E21">
+      <c r="E21" s="2">
         <v>44080.3</v>
       </c>
       <c r="F21" t="s">
@@ -1707,7 +1727,7 @@
       <c r="D22" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E22">
+      <c r="E22" s="2">
         <v>19555.71</v>
       </c>
       <c r="F22" t="s">
@@ -1733,7 +1753,7 @@
       <c r="D23" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E23">
+      <c r="E23" s="2">
         <v>12780.65</v>
       </c>
       <c r="F23" t="s">
@@ -1762,7 +1782,7 @@
       <c r="D24" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="2">
         <v>6802</v>
       </c>
       <c r="F24" t="s">
@@ -1791,7 +1811,7 @@
       <c r="D25" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E25">
+      <c r="E25" s="2">
         <v>18278.099999999999</v>
       </c>
       <c r="F25" t="s">
@@ -1820,7 +1840,7 @@
       <c r="D26" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E26">
+      <c r="E26" s="2">
         <v>42760.62</v>
       </c>
       <c r="F26" t="s">
@@ -1849,7 +1869,7 @@
       <c r="D27" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E27">
+      <c r="E27" s="2">
         <v>5906</v>
       </c>
       <c r="F27" t="s">
@@ -1878,7 +1898,7 @@
       <c r="D28" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E28">
+      <c r="E28" s="2">
         <v>5349</v>
       </c>
       <c r="F28" t="s">
@@ -1907,7 +1927,7 @@
       <c r="D29" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E29">
+      <c r="E29" s="2">
         <v>21699.54</v>
       </c>
       <c r="F29" t="s">
@@ -1933,7 +1953,7 @@
       <c r="D30" s="1">
         <v>45923</v>
       </c>
-      <c r="E30">
+      <c r="E30" s="2">
         <v>32566</v>
       </c>
       <c r="F30" t="s">
@@ -1959,7 +1979,7 @@
       <c r="D31" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E31">
+      <c r="E31" s="2">
         <v>12757.22</v>
       </c>
       <c r="F31" t="s">
@@ -1985,7 +2005,7 @@
       <c r="D32" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E32">
+      <c r="E32" s="2">
         <v>7137</v>
       </c>
       <c r="F32" t="s">
@@ -2008,7 +2028,7 @@
       <c r="D33" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E33">
+      <c r="E33" s="2">
         <v>16289.82</v>
       </c>
       <c r="F33" t="s">
@@ -2034,7 +2054,7 @@
       <c r="D34" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E34">
+      <c r="E34" s="2">
         <v>18817.400000000001</v>
       </c>
       <c r="F34" t="s">
@@ -2063,7 +2083,7 @@
       <c r="D35" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E35">
+      <c r="E35" s="2">
         <v>8834.0499999999993</v>
       </c>
       <c r="F35" t="s">
@@ -2092,7 +2112,7 @@
       <c r="D36" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E36">
+      <c r="E36" s="2">
         <v>12634</v>
       </c>
       <c r="F36" t="s">
@@ -2121,7 +2141,7 @@
       <c r="D37" s="1">
         <v>45972</v>
       </c>
-      <c r="E37">
+      <c r="E37" s="2">
         <v>17637.900000000001</v>
       </c>
       <c r="F37" t="s">
@@ -2147,7 +2167,7 @@
       <c r="D38" s="1">
         <v>45923</v>
       </c>
-      <c r="E38">
+      <c r="E38" s="2">
         <v>22541.05</v>
       </c>
       <c r="F38" t="s">
@@ -2173,7 +2193,7 @@
       <c r="D39" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="E39">
+      <c r="E39" s="2">
         <v>16955.25</v>
       </c>
       <c r="F39" t="s">
@@ -2199,7 +2219,7 @@
       <c r="D40" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E40">
+      <c r="E40" s="2">
         <v>21892.55</v>
       </c>
       <c r="F40" t="s">
@@ -2228,7 +2248,7 @@
       <c r="D41" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E41">
+      <c r="E41" s="2">
         <v>18892.650000000001</v>
       </c>
       <c r="F41" t="s">
@@ -2254,7 +2274,7 @@
       <c r="D42" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E42">
+      <c r="E42" s="2">
         <v>29888.25</v>
       </c>
       <c r="F42" t="s">
@@ -2283,7 +2303,7 @@
       <c r="D43" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E43">
+      <c r="E43" s="2">
         <v>17155.490000000002</v>
       </c>
       <c r="F43" t="s">
@@ -2312,7 +2332,7 @@
       <c r="D44" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E44">
+      <c r="E44" s="2">
         <v>6634.65</v>
       </c>
       <c r="F44" t="s">
@@ -2341,7 +2361,7 @@
       <c r="D45" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E45">
+      <c r="E45" s="2">
         <v>10856.55</v>
       </c>
       <c r="F45" t="s">
@@ -2370,7 +2390,7 @@
       <c r="D46" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="E46">
+      <c r="E46" s="2">
         <v>14729.21</v>
       </c>
       <c r="F46" t="s">
@@ -2399,7 +2419,7 @@
       <c r="D47" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E47">
+      <c r="E47" s="2">
         <v>5979.65</v>
       </c>
       <c r="F47" t="s">
@@ -2428,7 +2448,7 @@
       <c r="D48" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E48">
+      <c r="E48" s="2">
         <v>14749.35</v>
       </c>
       <c r="F48" t="s">
@@ -2457,7 +2477,7 @@
       <c r="D49" s="1">
         <v>45972</v>
       </c>
-      <c r="E49">
+      <c r="E49" s="2">
         <v>40800.050000000003</v>
       </c>
       <c r="F49" t="s">
@@ -2483,7 +2503,7 @@
       <c r="D50" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E50">
+      <c r="E50" s="2">
         <v>7025.18</v>
       </c>
       <c r="F50" t="s">
@@ -2512,7 +2532,7 @@
       <c r="D51" s="1">
         <v>45972</v>
       </c>
-      <c r="E51">
+      <c r="E51" s="2">
         <v>5800</v>
       </c>
       <c r="F51" t="s">
@@ -2538,7 +2558,7 @@
       <c r="D52" s="1">
         <v>45972</v>
       </c>
-      <c r="E52">
+      <c r="E52" s="2">
         <v>17816.099999999999</v>
       </c>
       <c r="F52" t="s">
@@ -2564,7 +2584,7 @@
       <c r="D53" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E53">
+      <c r="E53" s="2">
         <v>18072.7</v>
       </c>
       <c r="F53" t="s">
@@ -2593,7 +2613,7 @@
       <c r="D54" s="1">
         <v>45972</v>
       </c>
-      <c r="E54">
+      <c r="E54" s="2">
         <v>11960.5</v>
       </c>
       <c r="F54" t="s">
@@ -2619,7 +2639,7 @@
       <c r="D55" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E55">
+      <c r="E55" s="2">
         <v>19531.060000000001</v>
       </c>
       <c r="F55" t="s">
@@ -2648,7 +2668,7 @@
       <c r="D56" s="1">
         <v>45972</v>
       </c>
-      <c r="E56">
+      <c r="E56" s="2">
         <v>5987.19</v>
       </c>
       <c r="F56" t="s">
@@ -2674,7 +2694,7 @@
       <c r="D57" s="1">
         <v>45923</v>
       </c>
-      <c r="E57">
+      <c r="E57" s="2">
         <v>4920.2</v>
       </c>
       <c r="F57" t="s">
@@ -2697,7 +2717,7 @@
       <c r="D58" s="1">
         <v>45972</v>
       </c>
-      <c r="E58">
+      <c r="E58" s="2">
         <v>3823</v>
       </c>
       <c r="F58" t="s">
@@ -2720,7 +2740,7 @@
       <c r="D59" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E59">
+      <c r="E59" s="2">
         <v>11177.85</v>
       </c>
       <c r="F59" t="s">
@@ -2749,7 +2769,7 @@
       <c r="D60" s="1">
         <v>45923</v>
       </c>
-      <c r="E60">
+      <c r="E60" s="2">
         <v>11013.73</v>
       </c>
       <c r="F60" t="s">
@@ -2775,7 +2795,7 @@
       <c r="D61" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E61">
+      <c r="E61" s="2">
         <v>15382.85</v>
       </c>
       <c r="F61" t="s">
@@ -2804,7 +2824,7 @@
       <c r="D62" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="E62">
+      <c r="E62" s="2">
         <v>16637.5</v>
       </c>
       <c r="F62" t="s">
@@ -2833,7 +2853,7 @@
       <c r="D63" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E63">
+      <c r="E63" s="2">
         <v>16632.54</v>
       </c>
       <c r="F63" t="s">
@@ -2862,7 +2882,7 @@
       <c r="D64" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E64">
+      <c r="E64" s="2">
         <v>29455.49</v>
       </c>
       <c r="F64" t="s">
@@ -2891,7 +2911,7 @@
       <c r="D65" s="1">
         <v>45923</v>
       </c>
-      <c r="E65">
+      <c r="E65" s="2">
         <v>8125</v>
       </c>
       <c r="F65" t="s">
@@ -2914,7 +2934,7 @@
       <c r="D66" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E66">
+      <c r="E66" s="2">
         <v>6320</v>
       </c>
       <c r="F66" t="s">
@@ -2943,7 +2963,7 @@
       <c r="D67" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E67">
+      <c r="E67" s="2">
         <v>16750</v>
       </c>
       <c r="F67" t="s">
@@ -2972,7 +2992,7 @@
       <c r="D68" s="1">
         <v>45974</v>
       </c>
-      <c r="E68">
+      <c r="E68" s="2">
         <v>27961.54</v>
       </c>
       <c r="F68" t="s">
@@ -2998,7 +3018,7 @@
       <c r="D69" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E69">
+      <c r="E69" s="2">
         <v>19302.03</v>
       </c>
       <c r="F69" t="s">
@@ -3027,7 +3047,7 @@
       <c r="D70" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E70">
+      <c r="E70" s="2">
         <v>12823.87</v>
       </c>
       <c r="F70" t="s">
@@ -3038,267 +3058,268 @@
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A71" s="2" t="s">
+      <c r="A71" t="s">
         <v>218</v>
       </c>
-      <c r="B71" s="2" t="s">
+      <c r="B71" t="s">
         <v>219</v>
       </c>
-      <c r="C71" s="2">
+      <c r="C71">
         <v>23358</v>
       </c>
-      <c r="D71" s="3" t="s">
+      <c r="D71" s="1" t="s">
         <v>220</v>
       </c>
       <c r="E71" s="2">
         <v>15585.35</v>
       </c>
-      <c r="F71" s="2" t="s">
+      <c r="F71" t="s">
         <v>221</v>
       </c>
-      <c r="G71" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H71" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I71" s="2" t="s">
+      <c r="G71" t="s">
+        <v>13</v>
+      </c>
+      <c r="H71" t="s">
+        <v>13</v>
+      </c>
+      <c r="I71" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A72" s="2" t="s">
+      <c r="A72" t="s">
         <v>222</v>
       </c>
-      <c r="B72" s="2" t="s">
+      <c r="B72" t="s">
         <v>223</v>
       </c>
-      <c r="C72" s="2">
+      <c r="C72">
         <v>23359</v>
       </c>
-      <c r="D72" s="3" t="s">
+      <c r="D72" s="1" t="s">
         <v>220</v>
       </c>
       <c r="E72" s="2">
         <v>13421.04</v>
       </c>
-      <c r="F72" s="2" t="s">
+      <c r="F72" t="s">
         <v>224</v>
       </c>
-      <c r="G72" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H72" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I72" s="2" t="s">
+      <c r="G72" t="s">
+        <v>13</v>
+      </c>
+      <c r="H72" t="s">
+        <v>13</v>
+      </c>
+      <c r="I72" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A73" s="2" t="s">
+      <c r="A73" t="s">
         <v>225</v>
       </c>
-      <c r="B73" s="2" t="s">
+      <c r="B73" t="s">
         <v>226</v>
       </c>
-      <c r="C73" s="2">
+      <c r="C73">
         <v>23360</v>
       </c>
-      <c r="D73" s="3" t="s">
+      <c r="D73" s="1" t="s">
         <v>220</v>
       </c>
       <c r="E73" s="2">
         <v>8684.85</v>
       </c>
-      <c r="F73" s="2" t="s">
+      <c r="F73" t="s">
         <v>151</v>
       </c>
-      <c r="G73" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H73" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I73" s="2" t="s">
+      <c r="G73" t="s">
+        <v>13</v>
+      </c>
+      <c r="H73" t="s">
+        <v>13</v>
+      </c>
+      <c r="I73" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A74" s="2" t="s">
+      <c r="A74" t="s">
         <v>227</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B74" t="s">
         <v>228</v>
       </c>
-      <c r="C74" s="2">
+      <c r="C74">
         <v>23361</v>
       </c>
-      <c r="D74" s="3" t="s">
+      <c r="D74" s="1" t="s">
         <v>220</v>
       </c>
       <c r="E74" s="2">
         <v>23112.7</v>
       </c>
-      <c r="F74" s="2" t="s">
+      <c r="F74" t="s">
         <v>229</v>
       </c>
-      <c r="G74" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H74" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I74" s="2" t="s">
+      <c r="G74" t="s">
+        <v>13</v>
+      </c>
+      <c r="H74" t="s">
+        <v>13</v>
+      </c>
+      <c r="I74" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A75" s="2" t="s">
+      <c r="A75" t="s">
         <v>230</v>
       </c>
-      <c r="B75" s="2" t="s">
+      <c r="B75" t="s">
         <v>231</v>
       </c>
-      <c r="C75" s="2">
+      <c r="C75">
         <v>23362</v>
       </c>
-      <c r="D75" s="3" t="s">
+      <c r="D75" s="1" t="s">
         <v>220</v>
       </c>
       <c r="E75" s="2">
         <v>21247.85</v>
       </c>
-      <c r="F75" s="2" t="s">
+      <c r="F75" t="s">
         <v>232</v>
       </c>
-      <c r="G75" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H75" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I75" s="2" t="s">
+      <c r="G75" t="s">
+        <v>13</v>
+      </c>
+      <c r="H75" t="s">
+        <v>13</v>
+      </c>
+      <c r="I75" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A76" s="2" t="s">
+      <c r="A76" t="s">
         <v>233</v>
       </c>
-      <c r="B76" s="2" t="s">
+      <c r="B76" t="s">
         <v>234</v>
       </c>
-      <c r="C76" s="2">
+      <c r="C76">
         <v>23363</v>
       </c>
-      <c r="D76" s="3" t="s">
+      <c r="D76" s="1" t="s">
         <v>220</v>
       </c>
       <c r="E76" s="2">
         <v>18253.009999999998</v>
       </c>
-      <c r="F76" s="2" t="s">
+      <c r="F76" t="s">
         <v>235</v>
       </c>
-      <c r="G76" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H76" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I76" s="2" t="s">
+      <c r="G76" t="s">
+        <v>13</v>
+      </c>
+      <c r="H76" t="s">
+        <v>13</v>
+      </c>
+      <c r="I76" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A77" s="2" t="s">
+      <c r="A77" t="s">
         <v>236</v>
       </c>
-      <c r="B77" s="2" t="s">
+      <c r="B77" t="s">
         <v>237</v>
       </c>
-      <c r="C77" s="2">
+      <c r="C77">
         <v>23364</v>
       </c>
-      <c r="D77" s="3" t="s">
+      <c r="D77" s="1" t="s">
         <v>220</v>
       </c>
       <c r="E77" s="2">
         <v>8320</v>
       </c>
-      <c r="F77" s="2" t="s">
+      <c r="F77" t="s">
         <v>238</v>
       </c>
-      <c r="G77" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H77" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I77" s="2" t="s">
+      <c r="G77" t="s">
+        <v>13</v>
+      </c>
+      <c r="H77" t="s">
+        <v>13</v>
+      </c>
+      <c r="I77" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A78" s="2" t="s">
+      <c r="A78" t="s">
         <v>239</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="B78" t="s">
         <v>240</v>
       </c>
-      <c r="C78" s="2">
+      <c r="C78">
         <v>23365</v>
       </c>
-      <c r="D78" s="3" t="s">
+      <c r="D78" s="1" t="s">
         <v>220</v>
       </c>
       <c r="E78" s="2">
         <v>5937</v>
       </c>
-      <c r="F78" s="2" t="s">
+      <c r="F78" t="s">
         <v>241</v>
       </c>
-      <c r="G78" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H78" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I78" s="2" t="s">
+      <c r="G78" t="s">
+        <v>13</v>
+      </c>
+      <c r="H78" t="s">
+        <v>13</v>
+      </c>
+      <c r="I78" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A79" s="2" t="s">
+      <c r="A79" t="s">
         <v>242</v>
       </c>
-      <c r="B79" s="2" t="s">
+      <c r="B79" t="s">
         <v>243</v>
       </c>
-      <c r="C79" s="2">
+      <c r="C79">
         <v>23366</v>
       </c>
-      <c r="D79" s="3" t="s">
+      <c r="D79" s="1" t="s">
         <v>220</v>
       </c>
       <c r="E79" s="2">
         <v>8922.09</v>
       </c>
-      <c r="F79" s="2" t="s">
+      <c r="F79" t="s">
         <v>244</v>
       </c>
-      <c r="G79" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H79" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I79" s="2" t="s">
+      <c r="G79" t="s">
+        <v>13</v>
+      </c>
+      <c r="H79" t="s">
+        <v>13</v>
+      </c>
+      <c r="I79" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>